<commit_message>
Updated shiji with amends and pictures by 2026-06-30
</commit_message>
<xml_diff>
--- a/blog/data/shiji.xlsx
+++ b/blog/data/shiji.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2" conformance="strict">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr dateCompatibility="0" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jasonzhu/gh/dockerian/poetry/blog/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jasonzhu/gh/dockerian/poetry/blog/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{9034640B-7E64-CF4D-800F-AEFE8869D287}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{B1BD4AE8-9D1A-8742-8C21-355F7E6248C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6900" yWindow="620" windowWidth="26920" windowHeight="21260" xr2:uid="{035C77B4-2818-3C48-B742-D782783FD081}"/>
   </bookViews>
@@ -25,7 +25,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="18" r:id="rId4"/>
+    <pivotCache cacheId="59" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="1139" uniqueCount="324">
+<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="1143" uniqueCount="326">
   <si>
     <t>APR</t>
   </si>
@@ -3455,10 +3455,6 @@
     <t>书评之当代言情小说</t>
   </si>
   <si>
-    <t>乙巳年春题记</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>⒊</t>
   </si>
   <si>
@@ -3477,6 +3473,18 @@
   </si>
   <si>
     <t>论毛词</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>初春小住随笔</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>七绝</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>旅途小记</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -3712,9 +3720,6 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3724,11 +3729,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="159">
+  <dxfs count="231">
     <dxf>
       <alignment horizontal="center"/>
     </dxf>
@@ -4093,9 +4101,78 @@
       <alignment horizontal="center" indent="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="left"/>
     </dxf>
     <dxf>
+      <alignment horizontal="left"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="center"/>
     </dxf>
     <dxf>
@@ -4160,6 +4237,153 @@
     </dxf>
     <dxf>
       <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" indent="0"/>
     </dxf>
     <dxf>
       <font>
@@ -4903,7 +5127,7 @@
                   <c:v>31</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>4</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5374,7 +5598,7 @@
                   <c:v>84</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>145</c:v>
+                  <c:v>147</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5715,7 +5939,7 @@
                   <c:v>109</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>59</c:v>
+                  <c:v>61</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>51</c:v>
@@ -6212,7 +6436,7 @@
                   <c:v>10</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>12</c:v>
+                  <c:v>14</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>15</c:v>
@@ -6487,9 +6711,9 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Jason Zhu" refreshedDateIso="2026-06-30T05:36:56.28000021446495925" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="220" xr:uid="{F177C5F1-7A94-314A-98B6-EAB71221BA53}">
+<pivotCacheDefinition xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Jason Zhu" refreshedDateIso="2026-06-30T06:04:21.55000019352883050" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="221" xr:uid="{5241C904-63A7-3D4A-99BD-468495537955}">
   <cacheSource type="worksheet">
-    <worksheetSource ref="A1:K221" sheet="mulu"/>
+    <worksheetSource ref="A1:K222" sheet="mulu"/>
   </cacheSource>
   <cacheFields count="11">
     <cacheField name="#" numFmtId="0">
@@ -6625,7 +6849,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheRecords xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="220">
+<pivotCacheRecords xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="221">
   <r>
     <x v="0"/>
     <s v="律诗"/>
@@ -9451,11 +9675,24 @@
     <x v="0"/>
     <s v="律诗"/>
     <s v="七律"/>
-    <s v="乙巳年春题记"/>
+    <s v="初春小住随笔"/>
     <x v="40"/>
     <s v="⒊"/>
     <x v="10"/>
     <x v="10"/>
+    <x v="0"/>
+    <m/>
+    <x v="5"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <s v="律诗"/>
+    <s v="七绝"/>
+    <s v="旅途小记"/>
+    <x v="40"/>
+    <s v="⒌"/>
+    <x v="5"/>
+    <x v="5"/>
     <x v="0"/>
     <m/>
     <x v="5"/>
@@ -9490,7 +9727,579 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{ABD62A81-D21F-AF40-9887-256A2371C827}" name="Year-Month" cacheId="18" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Year / Month" colHeaderCaption="Count">
+<pivotTableDefinition xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D81E2A36-B4D4-C64A-8916-5F26EC917766}" name="GroupByYear" cacheId="59" dataOnRows="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Data" updatedVersion="8" minRefreshableVersion="3" showMemberPropertyTips="0" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" gridDropZones="1" chartFormat="7">
+  <location ref="D1:E44" firstHeaderRow="2" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="11">
+    <pivotField dataField="1" compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
+    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
+    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
+    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
+    <pivotField axis="axisRow" compact="0" outline="0" showAll="0" includeNewItemsInFilter="1">
+      <items count="42">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item x="15"/>
+        <item x="16"/>
+        <item x="17"/>
+        <item x="18"/>
+        <item x="19"/>
+        <item x="20"/>
+        <item x="21"/>
+        <item x="22"/>
+        <item x="23"/>
+        <item x="24"/>
+        <item x="25"/>
+        <item x="26"/>
+        <item x="27"/>
+        <item x="28"/>
+        <item x="29"/>
+        <item x="30"/>
+        <item x="31"/>
+        <item x="32"/>
+        <item x="33"/>
+        <item x="34"/>
+        <item x="35"/>
+        <item x="36"/>
+        <item x="37"/>
+        <item x="38"/>
+        <item x="39"/>
+        <item x="40"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
+    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
+    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
+    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
+    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
+    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="4"/>
+  </rowFields>
+  <rowItems count="42">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="11"/>
+    </i>
+    <i>
+      <x v="12"/>
+    </i>
+    <i>
+      <x v="13"/>
+    </i>
+    <i>
+      <x v="14"/>
+    </i>
+    <i>
+      <x v="15"/>
+    </i>
+    <i>
+      <x v="16"/>
+    </i>
+    <i>
+      <x v="17"/>
+    </i>
+    <i>
+      <x v="18"/>
+    </i>
+    <i>
+      <x v="19"/>
+    </i>
+    <i>
+      <x v="20"/>
+    </i>
+    <i>
+      <x v="21"/>
+    </i>
+    <i>
+      <x v="22"/>
+    </i>
+    <i>
+      <x v="23"/>
+    </i>
+    <i>
+      <x v="24"/>
+    </i>
+    <i>
+      <x v="25"/>
+    </i>
+    <i>
+      <x v="26"/>
+    </i>
+    <i>
+      <x v="27"/>
+    </i>
+    <i>
+      <x v="28"/>
+    </i>
+    <i>
+      <x v="29"/>
+    </i>
+    <i>
+      <x v="30"/>
+    </i>
+    <i>
+      <x v="31"/>
+    </i>
+    <i>
+      <x v="32"/>
+    </i>
+    <i>
+      <x v="33"/>
+    </i>
+    <i>
+      <x v="34"/>
+    </i>
+    <i>
+      <x v="35"/>
+    </i>
+    <i>
+      <x v="36"/>
+    </i>
+    <i>
+      <x v="37"/>
+    </i>
+    <i>
+      <x v="38"/>
+    </i>
+    <i>
+      <x v="39"/>
+    </i>
+    <i>
+      <x v="40"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Group By Year" fld="0" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="2">
+    <format dxfId="145">
+      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="144">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+  </formats>
+  <chartFormats count="5">
+    <chartFormat chart="0" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="35"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="2">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="37"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="3">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="39"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="4">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="4" count="1" selected="0">
+            <x v="40"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16 EnabledSubtotalsDefault="0" SubtotalsOnTopDefault="0"/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B98A0D15-DB1D-EA44-8425-4A227615CAA2}" name="GroupBySeasons" cacheId="59" dataOnRows="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Data" updatedVersion="8" minRefreshableVersion="3" showMemberPropertyTips="0" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" gridDropZones="1">
+  <location ref="G1:H7" firstHeaderRow="2" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="11">
+    <pivotField dataField="1" compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
+    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
+    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
+    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
+    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
+    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
+    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
+    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
+    <pivotField axis="axisRow" compact="0" outline="0" showAll="0" includeNewItemsInFilter="1">
+      <items count="5">
+        <item x="1"/>
+        <item x="0"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
+    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="8"/>
+  </rowFields>
+  <rowItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="By Seasons" fld="0" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="7">
+    <format dxfId="152">
+      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="151">
+      <pivotArea outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="150">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="149">
+      <pivotArea field="8" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="148">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="8" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="147">
+      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="146">
+      <pivotArea type="topEnd" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+  </formats>
+  <pivotTableStyleInfo showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16 EnabledSubtotalsDefault="0" SubtotalsOnTopDefault="0"/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00C213C8-ABF5-044A-A69F-044CDE187BB0}" name="GroupByYears" cacheId="59" dataOnRows="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Data" updatedVersion="8" minRefreshableVersion="3" showMemberPropertyTips="0" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" gridDropZones="1">
+  <location ref="G29:H37" firstHeaderRow="2" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="11">
+    <pivotField dataField="1" compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
+    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
+    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
+    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
+    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
+    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
+    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
+    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
+    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
+    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
+    <pivotField axis="axisRow" compact="0" outline="0" showAll="0" includeNewItemsInFilter="1">
+      <items count="7">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="10"/>
+  </rowFields>
+  <rowItems count="7">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="By Years" fld="0" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="7">
+    <format dxfId="159">
+      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="158">
+      <pivotArea outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="157">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="156">
+      <pivotArea field="10" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="155">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="10" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="154">
+      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="153">
+      <pivotArea type="topEnd" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+  </formats>
+  <pivotTableStyleInfo showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16 EnabledSubtotalsDefault="0" SubtotalsOnTopDefault="0"/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{AF506FF1-37AE-D146-9F90-8EFE7EACE91F}" name="PivotTable3" cacheId="59" dataOnRows="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Data" updatedVersion="8" minRefreshableVersion="3" showMemberPropertyTips="0" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" gridDropZones="1">
+  <location ref="G9:H23" firstHeaderRow="2" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="11">
+    <pivotField dataField="1" compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
+    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
+    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
+    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
+    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
+    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
+    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
+    <pivotField axis="axisRow" compact="0" outline="0" showAll="0" includeNewItemsInFilter="1">
+      <items count="13">
+        <item x="6"/>
+        <item x="4"/>
+        <item x="10"/>
+        <item x="0"/>
+        <item x="5"/>
+        <item x="8"/>
+        <item x="11"/>
+        <item x="2"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item x="7"/>
+        <item x="9"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
+    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
+    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="7"/>
+  </rowFields>
+  <rowItems count="13">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="11"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="By Months" fld="0" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="7">
+    <format dxfId="166">
+      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="165">
+      <pivotArea outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="164">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="163">
+      <pivotArea field="7" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="162">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="7" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="161">
+      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="160">
+      <pivotArea type="topEnd" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+  </formats>
+  <pivotTableStyleInfo showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16 EnabledSubtotalsDefault="0" SubtotalsOnTopDefault="0"/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5EA7A02F-5151-DD4F-ACDC-173BA86287DE}" name="Year-Month" cacheId="59" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Year / Month" colHeaderCaption="Count">
   <location ref="A1:B43" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="11">
     <pivotField dataField="1" showAll="0">
@@ -9718,35 +10527,35 @@
     <dataField name="Count" fld="0" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="49">
-    <format dxfId="120">
+    <format dxfId="215">
       <pivotArea type="all" dataOnly="0" outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="119">
+    <format dxfId="214">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="118">
+    <format dxfId="213">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="117">
+    <format dxfId="212">
       <pivotArea field="0" type="button" dataOnly="0" labelOnly="1" outline="0"/>
     </format>
-    <format dxfId="116">
+    <format dxfId="211">
       <pivotArea type="topEnd" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="115">
+    <format dxfId="210">
       <pivotArea field="4" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="114">
+    <format dxfId="209">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="4" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="113">
+    <format dxfId="208">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="112">
+    <format dxfId="207">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="4" count="1" selected="0">
@@ -9759,7 +10568,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="111">
+    <format dxfId="206">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="4" count="1" selected="0">
@@ -9771,7 +10580,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="110">
+    <format dxfId="205">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="4" count="1" selected="0">
@@ -9784,7 +10593,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="109">
+    <format dxfId="204">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="4" count="1" selected="0">
@@ -9798,7 +10607,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="108">
+    <format dxfId="203">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="4" count="1" selected="0">
@@ -9811,7 +10620,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="107">
+    <format dxfId="202">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="4" count="1" selected="0">
@@ -9825,7 +10634,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="106">
+    <format dxfId="201">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="4" count="1" selected="0">
@@ -9838,7 +10647,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="105">
+    <format dxfId="200">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="4" count="1" selected="0">
@@ -9851,7 +10660,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="104">
+    <format dxfId="199">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="4" count="1" selected="0">
@@ -9863,7 +10672,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="103">
+    <format dxfId="198">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="4" count="1" selected="0">
@@ -9876,7 +10685,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="102">
+    <format dxfId="197">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="4" count="1" selected="0">
@@ -9888,7 +10697,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="101">
+    <format dxfId="196">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="4" count="1" selected="0">
@@ -9900,7 +10709,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="100">
+    <format dxfId="195">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="4" count="1" selected="0">
@@ -9915,7 +10724,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="99">
+    <format dxfId="194">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="4" count="1" selected="0">
@@ -9932,7 +10741,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="98">
+    <format dxfId="193">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="4" count="1" selected="0">
@@ -9945,7 +10754,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="97">
+    <format dxfId="192">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="4" count="1" selected="0">
@@ -9957,7 +10766,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="96">
+    <format dxfId="191">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="4" count="1" selected="0">
@@ -9969,7 +10778,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="95">
+    <format dxfId="190">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="4" count="1" selected="0">
@@ -9981,7 +10790,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="94">
+    <format dxfId="189">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="4" count="1" selected="0">
@@ -9993,7 +10802,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="93">
+    <format dxfId="188">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="4" count="1" selected="0">
@@ -10006,7 +10815,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="92">
+    <format dxfId="187">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="4" count="1" selected="0">
@@ -10021,7 +10830,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="91">
+    <format dxfId="186">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="4" count="1" selected="0">
@@ -10034,7 +10843,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="90">
+    <format dxfId="185">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="4" count="1" selected="0">
@@ -10048,7 +10857,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="89">
+    <format dxfId="184">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="4" count="1" selected="0">
@@ -10062,7 +10871,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="88">
+    <format dxfId="183">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="4" count="1" selected="0">
@@ -10078,7 +10887,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="87">
+    <format dxfId="182">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="4" count="1" selected="0">
@@ -10094,7 +10903,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="86">
+    <format dxfId="181">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="4" count="1" selected="0">
@@ -10107,7 +10916,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="85">
+    <format dxfId="180">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="4" count="1" selected="0">
@@ -10119,7 +10928,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="84">
+    <format dxfId="179">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="4" count="1" selected="0">
@@ -10137,7 +10946,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="83">
+    <format dxfId="178">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="4" count="1" selected="0">
@@ -10151,7 +10960,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="82">
+    <format dxfId="177">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="4" count="1" selected="0">
@@ -10165,7 +10974,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="81">
+    <format dxfId="176">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="4" count="1" selected="0">
@@ -10179,7 +10988,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="80">
+    <format dxfId="175">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="4" count="1" selected="0">
@@ -10191,7 +11000,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="79">
+    <format dxfId="174">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="4" count="1" selected="0">
@@ -10203,7 +11012,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="78">
+    <format dxfId="173">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="4" count="1" selected="0">
@@ -10217,7 +11026,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="77">
+    <format dxfId="172">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="4" count="1" selected="0">
@@ -10238,7 +11047,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="76">
+    <format dxfId="171">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="4" count="1" selected="0">
@@ -10255,7 +11064,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="75">
+    <format dxfId="170">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="4" count="1" selected="0">
@@ -10274,7 +11083,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="74">
+    <format dxfId="169">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="4" count="1" selected="0">
@@ -10291,7 +11100,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="73">
+    <format dxfId="168">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="2">
           <reference field="4" count="1" selected="0">
@@ -10311,7 +11120,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="72">
+    <format dxfId="167">
       <pivotArea dataOnly="0" labelOnly="1" grandCol="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -10324,593 +11133,21 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{614E86C4-F4E7-E942-9280-99870EBBE403}" name="GroupByYear" cacheId="18" dataOnRows="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Data" updatedVersion="8" minRefreshableVersion="3" showMemberPropertyTips="0" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" gridDropZones="1" chartFormat="7">
-  <location ref="D1:E44" firstHeaderRow="2" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="11">
-    <pivotField dataField="1" compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField axis="axisRow" compact="0" outline="0" showAll="0" includeNewItemsInFilter="1">
-      <items count="42">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item x="9"/>
-        <item x="10"/>
-        <item x="11"/>
-        <item x="12"/>
-        <item x="13"/>
-        <item x="14"/>
-        <item x="15"/>
-        <item x="16"/>
-        <item x="17"/>
-        <item x="18"/>
-        <item x="19"/>
-        <item x="20"/>
-        <item x="21"/>
-        <item x="22"/>
-        <item x="23"/>
-        <item x="24"/>
-        <item x="25"/>
-        <item x="26"/>
-        <item x="27"/>
-        <item x="28"/>
-        <item x="29"/>
-        <item x="30"/>
-        <item x="31"/>
-        <item x="32"/>
-        <item x="33"/>
-        <item x="34"/>
-        <item x="35"/>
-        <item x="36"/>
-        <item x="37"/>
-        <item x="38"/>
-        <item x="39"/>
-        <item x="40"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="4"/>
-  </rowFields>
-  <rowItems count="42">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="8"/>
-    </i>
-    <i>
-      <x v="9"/>
-    </i>
-    <i>
-      <x v="10"/>
-    </i>
-    <i>
-      <x v="11"/>
-    </i>
-    <i>
-      <x v="12"/>
-    </i>
-    <i>
-      <x v="13"/>
-    </i>
-    <i>
-      <x v="14"/>
-    </i>
-    <i>
-      <x v="15"/>
-    </i>
-    <i>
-      <x v="16"/>
-    </i>
-    <i>
-      <x v="17"/>
-    </i>
-    <i>
-      <x v="18"/>
-    </i>
-    <i>
-      <x v="19"/>
-    </i>
-    <i>
-      <x v="20"/>
-    </i>
-    <i>
-      <x v="21"/>
-    </i>
-    <i>
-      <x v="22"/>
-    </i>
-    <i>
-      <x v="23"/>
-    </i>
-    <i>
-      <x v="24"/>
-    </i>
-    <i>
-      <x v="25"/>
-    </i>
-    <i>
-      <x v="26"/>
-    </i>
-    <i>
-      <x v="27"/>
-    </i>
-    <i>
-      <x v="28"/>
-    </i>
-    <i>
-      <x v="29"/>
-    </i>
-    <i>
-      <x v="30"/>
-    </i>
-    <i>
-      <x v="31"/>
-    </i>
-    <i>
-      <x v="32"/>
-    </i>
-    <i>
-      <x v="33"/>
-    </i>
-    <i>
-      <x v="34"/>
-    </i>
-    <i>
-      <x v="35"/>
-    </i>
-    <i>
-      <x v="36"/>
-    </i>
-    <i>
-      <x v="37"/>
-    </i>
-    <i>
-      <x v="38"/>
-    </i>
-    <i>
-      <x v="39"/>
-    </i>
-    <i>
-      <x v="40"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Group By Year" fld="0" baseField="0" baseItem="0"/>
-  </dataFields>
-  <formats count="2">
-    <format dxfId="122">
-      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="121">
-      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-  </formats>
-  <chartFormats count="5">
-    <chartFormat chart="0" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="0" format="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="35"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="0" format="2">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="37"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="0" format="3">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="39"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="0" format="4">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="4" count="1" selected="0">
-            <x v="40"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16 EnabledSubtotalsDefault="0" SubtotalsOnTopDefault="0"/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{380DFDF7-75FA-7B49-824A-260966BA644F}" name="GroupBySeasons" cacheId="18" dataOnRows="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Data" updatedVersion="8" minRefreshableVersion="3" showMemberPropertyTips="0" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" gridDropZones="1">
-  <location ref="G1:H7" firstHeaderRow="2" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="11">
-    <pivotField dataField="1" compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField axis="axisRow" compact="0" outline="0" showAll="0" includeNewItemsInFilter="1">
-      <items count="5">
-        <item x="1"/>
-        <item x="0"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="8"/>
-  </rowFields>
-  <rowItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="By Seasons" fld="0" baseField="0" baseItem="0"/>
-  </dataFields>
-  <formats count="7">
-    <format dxfId="129">
-      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="128">
-      <pivotArea outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="127">
-      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="126">
-      <pivotArea field="8" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
-    </format>
-    <format dxfId="125">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="8" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="124">
-      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="123">
-      <pivotArea type="topEnd" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-  </formats>
-  <pivotTableStyleInfo showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16 EnabledSubtotalsDefault="0" SubtotalsOnTopDefault="0"/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4A9269E0-89B1-D94B-8942-D8B7B921C3CD}" name="GroupByYears" cacheId="18" dataOnRows="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Data" updatedVersion="8" minRefreshableVersion="3" showMemberPropertyTips="0" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" gridDropZones="1">
-  <location ref="G29:H37" firstHeaderRow="2" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="11">
-    <pivotField dataField="1" compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField axis="axisRow" compact="0" outline="0" showAll="0" includeNewItemsInFilter="1">
-      <items count="7">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="10"/>
-  </rowFields>
-  <rowItems count="7">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="By Years" fld="0" baseField="0" baseItem="0"/>
-  </dataFields>
-  <formats count="7">
-    <format dxfId="136">
-      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="135">
-      <pivotArea outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="134">
-      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="133">
-      <pivotArea field="10" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
-    </format>
-    <format dxfId="132">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="10" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="131">
-      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="130">
-      <pivotArea type="topEnd" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-  </formats>
-  <pivotTableStyleInfo showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16 EnabledSubtotalsDefault="0" SubtotalsOnTopDefault="0"/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{66A8050B-09F0-9B4F-8805-EB201B9B0856}" name="PivotTable3" cacheId="18" dataOnRows="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Data" updatedVersion="8" minRefreshableVersion="3" showMemberPropertyTips="0" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" gridDropZones="1">
-  <location ref="G9:H23" firstHeaderRow="2" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="11">
-    <pivotField dataField="1" compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField axis="axisRow" compact="0" outline="0" showAll="0" includeNewItemsInFilter="1">
-      <items count="13">
-        <item x="6"/>
-        <item x="4"/>
-        <item x="10"/>
-        <item x="0"/>
-        <item x="5"/>
-        <item x="8"/>
-        <item x="11"/>
-        <item x="2"/>
-        <item x="1"/>
-        <item x="3"/>
-        <item x="7"/>
-        <item x="9"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
-    <pivotField compact="0" outline="0" showAll="0" includeNewItemsInFilter="1"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="7"/>
-  </rowFields>
-  <rowItems count="13">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="8"/>
-    </i>
-    <i>
-      <x v="9"/>
-    </i>
-    <i>
-      <x v="10"/>
-    </i>
-    <i>
-      <x v="11"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="By Months" fld="0" baseField="0" baseItem="0"/>
-  </dataFields>
-  <formats count="7">
-    <format dxfId="143">
-      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="142">
-      <pivotArea outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="141">
-      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="140">
-      <pivotArea field="7" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
-    </format>
-    <format dxfId="139">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="7" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="138">
-      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="137">
-      <pivotArea type="topEnd" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-  </formats>
-  <pivotTableStyleInfo showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16 EnabledSubtotalsDefault="0" SubtotalsOnTopDefault="0"/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FABD02-9A4F-2F4E-98CC-4A41CC9E9AD0}" name="Table2" displayName="Table2" ref="A1:K65539" totalsRowShown="0" headerRowDxfId="158" dataDxfId="156" headerRowBorderDxfId="157" tableBorderDxfId="155">
+<table xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FABD02-9A4F-2F4E-98CC-4A41CC9E9AD0}" name="Table2" displayName="Table2" ref="A1:K65539" totalsRowShown="0" headerRowDxfId="230" dataDxfId="228" headerRowBorderDxfId="229" tableBorderDxfId="227">
   <autoFilter ref="A1:K65539" xr:uid="{4C4B196D-BF96-E846-9447-43C2E95DA6FC}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="#" dataDxfId="154"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="分类" dataDxfId="153"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="格体" dataDxfId="152"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="标题" dataDxfId="151"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="年" dataDxfId="150"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="月份" dataDxfId="149"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="月" dataDxfId="148"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="Month" dataDxfId="147"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="Season" dataDxfId="146"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="S#" dataDxfId="145"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0100-00000B000000}" name="Years" dataDxfId="144"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="#" dataDxfId="226"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="分类" dataDxfId="225"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="格体" dataDxfId="224"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="标题" dataDxfId="223"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="年" dataDxfId="222"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="月份" dataDxfId="221"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="月" dataDxfId="220"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="Month" dataDxfId="219"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="Season" dataDxfId="218"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="S#" dataDxfId="217"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0100-00000B000000}" name="Years" dataDxfId="216"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -11233,7 +11470,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9ABD77E-50FB-F946-95D5-F5072752F13B}">
-  <dimension ref="A1:K221"/>
+  <dimension ref="A1:K222"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="25" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="5.83203125" style="2" customWidth="1"/>
@@ -18601,7 +18838,7 @@
         <v>3</v>
       </c>
       <c r="H194" s="2" t="str">
-        <f t="shared" ref="H194:H257" si="6">UPPER(TEXT(DATE(2026, G194, 1), "mmm"))</f>
+        <f t="shared" ref="H194:H221" si="6">UPPER(TEXT(DATE(2026, G194, 1), "mmm"))</f>
         <v>MAR</v>
       </c>
       <c r="I194" s="2" t="str">
@@ -18612,7 +18849,7 @@
         <v>290</v>
       </c>
       <c r="K194" s="2">
-        <f t="shared" ref="K194:K221" si="7">ROUNDDOWN(E194/10,0)*10</f>
+        <f t="shared" ref="K194:K222" si="7">ROUNDDOWN(E194/10,0)*10</f>
         <v>2020</v>
       </c>
     </row>
@@ -19530,19 +19767,19 @@
         <v>311</v>
       </c>
       <c r="D219" s="7" t="s">
-        <v>317</v>
+        <v>323</v>
       </c>
       <c r="E219" s="2">
         <v>2026</v>
       </c>
       <c r="F219" s="19" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="G219" s="2">
         <v>3</v>
       </c>
       <c r="H219" s="2" t="str">
-        <f t="shared" si="6"/>
+        <f>UPPER(TEXT(DATE(2026, G219, 1), "mmm"))</f>
         <v>MAR</v>
       </c>
       <c r="I219" s="2" t="str">
@@ -19556,28 +19793,28 @@
     </row>
     <row r="220" spans="1:11" ht="25" customHeight="1">
       <c r="A220" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B220" s="8" t="s">
         <v>310</v>
       </c>
       <c r="C220" s="7" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="D220" s="7" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="E220" s="2">
         <v>2026</v>
       </c>
       <c r="F220" s="19" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="G220" s="2">
         <v>5</v>
       </c>
       <c r="H220" s="2" t="str">
-        <f t="shared" si="6"/>
+        <f>UPPER(TEXT(DATE(2026, G220, 1), "mmm"))</f>
         <v>MAY</v>
       </c>
       <c r="I220" s="2" t="str">
@@ -19597,7 +19834,7 @@
         <v>310</v>
       </c>
       <c r="C221" s="7" t="s">
-        <v>311</v>
+        <v>320</v>
       </c>
       <c r="D221" s="7" t="s">
         <v>322</v>
@@ -19606,20 +19843,55 @@
         <v>2026</v>
       </c>
       <c r="F221" s="19" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="G221" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H221" s="2" t="str">
-        <f t="shared" si="6"/>
-        <v>JUN</v>
+        <f>UPPER(TEXT(DATE(2026, G221, 1), "mmm"))</f>
+        <v>MAY</v>
       </c>
       <c r="I221" s="2" t="str">
         <f>LOOKUP(G221,{1,3,6,9,12},{"Winter","Spring","Summer","Autumn","Winter"})</f>
+        <v>Spring</v>
+      </c>
+      <c r="K221" s="2">
+        <f t="shared" si="7"/>
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="222" spans="1:11" ht="25" customHeight="1">
+      <c r="A222" s="2">
+        <v>1</v>
+      </c>
+      <c r="B222" s="8" t="s">
+        <v>310</v>
+      </c>
+      <c r="C222" s="7" t="s">
+        <v>311</v>
+      </c>
+      <c r="D222" s="7" t="s">
+        <v>321</v>
+      </c>
+      <c r="E222" s="2">
+        <v>2026</v>
+      </c>
+      <c r="F222" s="19" t="s">
+        <v>319</v>
+      </c>
+      <c r="G222" s="2">
+        <v>6</v>
+      </c>
+      <c r="H222" s="2" t="str">
+        <f>UPPER(TEXT(DATE(2026, G222, 1), "mmm"))</f>
+        <v>JUN</v>
+      </c>
+      <c r="I222" s="2" t="str">
+        <f>LOOKUP(G222,{1,3,6,9,12},{"Winter","Spring","Summer","Autumn","Winter"})</f>
         <v>Summer</v>
       </c>
-      <c r="K221" s="2">
+      <c r="K222" s="2">
         <f t="shared" si="7"/>
         <v>2020</v>
       </c>
@@ -19649,7 +19921,7 @@
     <col min="4" max="4" width="14.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="6.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.83203125" style="1"/>
-    <col min="7" max="7" width="12.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.1640625" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="9" width="6.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="12.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="6.33203125" style="1" bestFit="1" customWidth="1"/>
@@ -19686,7 +19958,7 @@
       <c r="A2" s="1">
         <v>1979</v>
       </c>
-      <c r="B2" s="20">
+      <c r="B2" s="23">
         <v>4</v>
       </c>
       <c r="C2"/>
@@ -19716,21 +19988,21 @@
       <c r="A3" s="1">
         <v>1980</v>
       </c>
-      <c r="B3" s="20">
+      <c r="B3" s="23">
         <v>2</v>
       </c>
       <c r="C3"/>
       <c r="D3" s="10">
         <v>1979</v>
       </c>
-      <c r="E3" s="21">
+      <c r="E3" s="20">
         <v>4</v>
       </c>
       <c r="F3"/>
       <c r="G3" s="10" t="s">
         <v>302</v>
       </c>
-      <c r="H3" s="21">
+      <c r="H3" s="20">
         <v>109</v>
       </c>
       <c r="I3"/>
@@ -19746,22 +20018,22 @@
       <c r="A4" s="1">
         <v>1982</v>
       </c>
-      <c r="B4" s="20">
+      <c r="B4" s="23">
         <v>7</v>
       </c>
       <c r="C4"/>
       <c r="D4" s="11">
         <v>1980</v>
       </c>
-      <c r="E4" s="22">
+      <c r="E4" s="21">
         <v>2</v>
       </c>
       <c r="F4"/>
       <c r="G4" s="11" t="s">
         <v>303</v>
       </c>
-      <c r="H4" s="22">
-        <v>59</v>
+      <c r="H4" s="21">
+        <v>61</v>
       </c>
       <c r="I4"/>
       <c r="J4"/>
@@ -19776,21 +20048,21 @@
       <c r="A5" s="1">
         <v>1983</v>
       </c>
-      <c r="B5" s="20">
+      <c r="B5" s="23">
         <v>5</v>
       </c>
       <c r="C5"/>
       <c r="D5" s="11">
         <v>1982</v>
       </c>
-      <c r="E5" s="22">
+      <c r="E5" s="21">
         <v>7</v>
       </c>
       <c r="F5"/>
       <c r="G5" s="11" t="s">
         <v>304</v>
       </c>
-      <c r="H5" s="22">
+      <c r="H5" s="21">
         <v>51</v>
       </c>
       <c r="I5"/>
@@ -19806,21 +20078,21 @@
       <c r="A6" s="1">
         <v>1984</v>
       </c>
-      <c r="B6" s="20">
+      <c r="B6" s="23">
         <v>5</v>
       </c>
       <c r="C6"/>
       <c r="D6" s="11">
         <v>1983</v>
       </c>
-      <c r="E6" s="22">
+      <c r="E6" s="21">
         <v>5</v>
       </c>
       <c r="F6"/>
       <c r="G6" s="11" t="s">
         <v>305</v>
       </c>
-      <c r="H6" s="22">
+      <c r="H6" s="21">
         <v>124</v>
       </c>
       <c r="I6"/>
@@ -19836,22 +20108,22 @@
       <c r="A7" s="1">
         <v>1985</v>
       </c>
-      <c r="B7" s="20">
+      <c r="B7" s="23">
         <v>9</v>
       </c>
       <c r="C7"/>
       <c r="D7" s="11">
         <v>1984</v>
       </c>
-      <c r="E7" s="22">
+      <c r="E7" s="21">
         <v>5</v>
       </c>
       <c r="F7"/>
       <c r="G7" s="12" t="s">
         <v>284</v>
       </c>
-      <c r="H7" s="23">
-        <v>343</v>
+      <c r="H7" s="22">
+        <v>345</v>
       </c>
       <c r="I7"/>
       <c r="J7"/>
@@ -19866,14 +20138,14 @@
       <c r="A8" s="1">
         <v>1986</v>
       </c>
-      <c r="B8" s="20">
+      <c r="B8" s="23">
         <v>4</v>
       </c>
       <c r="C8"/>
       <c r="D8" s="11">
         <v>1985</v>
       </c>
-      <c r="E8" s="22">
+      <c r="E8" s="21">
         <v>9</v>
       </c>
       <c r="F8"/>
@@ -19892,14 +20164,14 @@
       <c r="A9" s="1">
         <v>1987</v>
       </c>
-      <c r="B9" s="20">
+      <c r="B9" s="23">
         <v>2</v>
       </c>
       <c r="C9"/>
       <c r="D9" s="11">
         <v>1986</v>
       </c>
-      <c r="E9" s="22">
+      <c r="E9" s="21">
         <v>4</v>
       </c>
       <c r="F9"/>
@@ -19920,14 +20192,14 @@
       <c r="A10" s="1">
         <v>1988</v>
       </c>
-      <c r="B10" s="20">
+      <c r="B10" s="23">
         <v>1</v>
       </c>
       <c r="C10"/>
       <c r="D10" s="11">
         <v>1987</v>
       </c>
-      <c r="E10" s="22">
+      <c r="E10" s="21">
         <v>2</v>
       </c>
       <c r="F10"/>
@@ -19950,21 +20222,21 @@
       <c r="A11" s="1">
         <v>1989</v>
       </c>
-      <c r="B11" s="20">
+      <c r="B11" s="23">
         <v>2</v>
       </c>
       <c r="C11"/>
       <c r="D11" s="11">
         <v>1988</v>
       </c>
-      <c r="E11" s="22">
+      <c r="E11" s="21">
         <v>1</v>
       </c>
       <c r="F11"/>
       <c r="G11" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="H11" s="21">
+      <c r="H11" s="20">
         <v>28</v>
       </c>
       <c r="I11"/>
@@ -19980,21 +20252,21 @@
       <c r="A12" s="1">
         <v>1992</v>
       </c>
-      <c r="B12" s="20">
+      <c r="B12" s="23">
         <v>1</v>
       </c>
       <c r="C12"/>
       <c r="D12" s="11">
         <v>1989</v>
       </c>
-      <c r="E12" s="22">
+      <c r="E12" s="21">
         <v>2</v>
       </c>
       <c r="F12"/>
       <c r="G12" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="H12" s="22">
+      <c r="H12" s="21">
         <v>63</v>
       </c>
       <c r="I12"/>
@@ -20010,21 +20282,21 @@
       <c r="A13" s="1">
         <v>1993</v>
       </c>
-      <c r="B13" s="20">
+      <c r="B13" s="23">
         <v>2</v>
       </c>
       <c r="C13"/>
       <c r="D13" s="11">
         <v>1992</v>
       </c>
-      <c r="E13" s="22">
+      <c r="E13" s="21">
         <v>1</v>
       </c>
       <c r="F13"/>
       <c r="G13" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="H13" s="22">
+      <c r="H13" s="21">
         <v>37</v>
       </c>
       <c r="I13"/>
@@ -20040,21 +20312,21 @@
       <c r="A14" s="1">
         <v>1994</v>
       </c>
-      <c r="B14" s="20">
+      <c r="B14" s="23">
         <v>8</v>
       </c>
       <c r="C14"/>
       <c r="D14" s="11">
         <v>1993</v>
       </c>
-      <c r="E14" s="22">
+      <c r="E14" s="21">
         <v>2</v>
       </c>
       <c r="F14"/>
       <c r="G14" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="H14" s="22">
+      <c r="H14" s="21">
         <v>10</v>
       </c>
       <c r="I14"/>
@@ -20070,22 +20342,22 @@
       <c r="A15" s="1">
         <v>1995</v>
       </c>
-      <c r="B15" s="20">
+      <c r="B15" s="23">
         <v>30</v>
       </c>
       <c r="C15"/>
       <c r="D15" s="11">
         <v>1994</v>
       </c>
-      <c r="E15" s="22">
+      <c r="E15" s="21">
         <v>8</v>
       </c>
       <c r="F15"/>
       <c r="G15" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="H15" s="22">
-        <v>12</v>
+      <c r="H15" s="21">
+        <v>14</v>
       </c>
       <c r="I15"/>
       <c r="J15"/>
@@ -20100,21 +20372,21 @@
       <c r="A16" s="1">
         <v>1996</v>
       </c>
-      <c r="B16" s="20">
+      <c r="B16" s="23">
         <v>2</v>
       </c>
       <c r="C16"/>
       <c r="D16" s="11">
         <v>1995</v>
       </c>
-      <c r="E16" s="22">
+      <c r="E16" s="21">
         <v>30</v>
       </c>
       <c r="F16"/>
       <c r="G16" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="H16" s="22">
+      <c r="H16" s="21">
         <v>15</v>
       </c>
       <c r="I16"/>
@@ -20130,21 +20402,21 @@
       <c r="A17" s="1">
         <v>1997</v>
       </c>
-      <c r="B17" s="20">
+      <c r="B17" s="23">
         <v>1</v>
       </c>
       <c r="C17"/>
       <c r="D17" s="11">
         <v>1996</v>
       </c>
-      <c r="E17" s="22">
+      <c r="E17" s="21">
         <v>2</v>
       </c>
       <c r="F17"/>
       <c r="G17" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="H17" s="22">
+      <c r="H17" s="21">
         <v>13</v>
       </c>
       <c r="I17"/>
@@ -20158,21 +20430,21 @@
       <c r="A18" s="1">
         <v>1998</v>
       </c>
-      <c r="B18" s="20">
+      <c r="B18" s="23">
         <v>1</v>
       </c>
       <c r="C18"/>
       <c r="D18" s="11">
         <v>1997</v>
       </c>
-      <c r="E18" s="22">
+      <c r="E18" s="21">
         <v>1</v>
       </c>
       <c r="F18"/>
       <c r="G18" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="H18" s="22">
+      <c r="H18" s="21">
         <v>23</v>
       </c>
       <c r="I18"/>
@@ -20186,21 +20458,21 @@
       <c r="A19" s="1">
         <v>1999</v>
       </c>
-      <c r="B19" s="20">
+      <c r="B19" s="23">
         <v>2</v>
       </c>
       <c r="C19"/>
       <c r="D19" s="11">
         <v>1998</v>
       </c>
-      <c r="E19" s="22">
+      <c r="E19" s="21">
         <v>1</v>
       </c>
       <c r="F19"/>
       <c r="G19" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="H19" s="22">
+      <c r="H19" s="21">
         <v>52</v>
       </c>
       <c r="I19"/>
@@ -20214,21 +20486,21 @@
       <c r="A20" s="1">
         <v>2002</v>
       </c>
-      <c r="B20" s="20">
+      <c r="B20" s="23">
         <v>1</v>
       </c>
       <c r="C20"/>
       <c r="D20" s="11">
         <v>1999</v>
       </c>
-      <c r="E20" s="22">
+      <c r="E20" s="21">
         <v>2</v>
       </c>
       <c r="F20"/>
       <c r="G20" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="H20" s="22">
+      <c r="H20" s="21">
         <v>25</v>
       </c>
       <c r="I20"/>
@@ -20242,21 +20514,21 @@
       <c r="A21" s="1">
         <v>2003</v>
       </c>
-      <c r="B21" s="20">
+      <c r="B21" s="23">
         <v>2</v>
       </c>
       <c r="C21"/>
       <c r="D21" s="11">
         <v>2002</v>
       </c>
-      <c r="E21" s="22">
+      <c r="E21" s="21">
         <v>1</v>
       </c>
       <c r="F21"/>
       <c r="G21" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="H21" s="22">
+      <c r="H21" s="21">
         <v>32</v>
       </c>
       <c r="I21"/>
@@ -20270,21 +20542,21 @@
       <c r="A22" s="1">
         <v>2006</v>
       </c>
-      <c r="B22" s="20">
+      <c r="B22" s="23">
         <v>6</v>
       </c>
       <c r="C22"/>
       <c r="D22" s="11">
         <v>2003</v>
       </c>
-      <c r="E22" s="22">
+      <c r="E22" s="21">
         <v>2</v>
       </c>
       <c r="F22"/>
       <c r="G22" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="H22" s="22">
+      <c r="H22" s="21">
         <v>33</v>
       </c>
       <c r="I22"/>
@@ -20298,22 +20570,22 @@
       <c r="A23" s="1">
         <v>2007</v>
       </c>
-      <c r="B23" s="20">
+      <c r="B23" s="23">
         <v>4</v>
       </c>
       <c r="C23"/>
       <c r="D23" s="11">
         <v>2006</v>
       </c>
-      <c r="E23" s="22">
+      <c r="E23" s="21">
         <v>6</v>
       </c>
       <c r="F23"/>
       <c r="G23" s="12" t="s">
         <v>284</v>
       </c>
-      <c r="H23" s="23">
-        <v>343</v>
+      <c r="H23" s="22">
+        <v>345</v>
       </c>
       <c r="I23"/>
       <c r="J23"/>
@@ -20326,14 +20598,14 @@
       <c r="A24" s="1">
         <v>2008</v>
       </c>
-      <c r="B24" s="20">
+      <c r="B24" s="23">
         <v>5</v>
       </c>
       <c r="C24"/>
       <c r="D24" s="11">
         <v>2007</v>
       </c>
-      <c r="E24" s="22">
+      <c r="E24" s="21">
         <v>4</v>
       </c>
       <c r="F24"/>
@@ -20350,14 +20622,14 @@
       <c r="A25" s="1">
         <v>2009</v>
       </c>
-      <c r="B25" s="20">
+      <c r="B25" s="23">
         <v>8</v>
       </c>
       <c r="C25"/>
       <c r="D25" s="11">
         <v>2008</v>
       </c>
-      <c r="E25" s="22">
+      <c r="E25" s="21">
         <v>5</v>
       </c>
       <c r="F25"/>
@@ -20370,14 +20642,14 @@
       <c r="A26" s="1">
         <v>2010</v>
       </c>
-      <c r="B26" s="20">
+      <c r="B26" s="23">
         <v>30</v>
       </c>
       <c r="C26"/>
       <c r="D26" s="11">
         <v>2009</v>
       </c>
-      <c r="E26" s="22">
+      <c r="E26" s="21">
         <v>8</v>
       </c>
       <c r="F26"/>
@@ -20390,14 +20662,14 @@
       <c r="A27" s="1">
         <v>2011</v>
       </c>
-      <c r="B27" s="20">
+      <c r="B27" s="23">
         <v>16</v>
       </c>
       <c r="C27"/>
       <c r="D27" s="11">
         <v>2010</v>
       </c>
-      <c r="E27" s="22">
+      <c r="E27" s="21">
         <v>30</v>
       </c>
       <c r="F27"/>
@@ -20410,14 +20682,14 @@
       <c r="A28" s="1">
         <v>2012</v>
       </c>
-      <c r="B28" s="20">
+      <c r="B28" s="23">
         <v>7</v>
       </c>
       <c r="C28"/>
       <c r="D28" s="11">
         <v>2011</v>
       </c>
-      <c r="E28" s="22">
+      <c r="E28" s="21">
         <v>16</v>
       </c>
       <c r="F28"/>
@@ -20430,14 +20702,14 @@
       <c r="A29" s="1">
         <v>2013</v>
       </c>
-      <c r="B29" s="20">
+      <c r="B29" s="23">
         <v>1</v>
       </c>
       <c r="C29"/>
       <c r="D29" s="11">
         <v>2012</v>
       </c>
-      <c r="E29" s="22">
+      <c r="E29" s="21">
         <v>7</v>
       </c>
       <c r="F29"/>
@@ -20456,14 +20728,14 @@
       <c r="A30" s="1">
         <v>2014</v>
       </c>
-      <c r="B30" s="20">
+      <c r="B30" s="23">
         <v>12</v>
       </c>
       <c r="C30"/>
       <c r="D30" s="11">
         <v>2013</v>
       </c>
-      <c r="E30" s="22">
+      <c r="E30" s="21">
         <v>1</v>
       </c>
       <c r="F30"/>
@@ -20484,21 +20756,21 @@
       <c r="A31" s="1">
         <v>2015</v>
       </c>
-      <c r="B31" s="20">
+      <c r="B31" s="23">
         <v>3</v>
       </c>
       <c r="C31"/>
       <c r="D31" s="11">
         <v>2014</v>
       </c>
-      <c r="E31" s="22">
+      <c r="E31" s="21">
         <v>12</v>
       </c>
       <c r="F31"/>
       <c r="G31" s="10">
         <v>1970</v>
       </c>
-      <c r="H31" s="21">
+      <c r="H31" s="20">
         <v>4</v>
       </c>
       <c r="I31"/>
@@ -20512,21 +20784,21 @@
       <c r="A32" s="1">
         <v>2016</v>
       </c>
-      <c r="B32" s="20">
+      <c r="B32" s="23">
         <v>5</v>
       </c>
       <c r="C32"/>
       <c r="D32" s="11">
         <v>2015</v>
       </c>
-      <c r="E32" s="22">
+      <c r="E32" s="21">
         <v>3</v>
       </c>
       <c r="F32"/>
       <c r="G32" s="11">
         <v>1980</v>
       </c>
-      <c r="H32" s="22">
+      <c r="H32" s="21">
         <v>37</v>
       </c>
       <c r="I32"/>
@@ -20540,21 +20812,21 @@
       <c r="A33" s="1">
         <v>2017</v>
       </c>
-      <c r="B33" s="20">
+      <c r="B33" s="23">
         <v>4</v>
       </c>
       <c r="C33"/>
       <c r="D33" s="11">
         <v>2016</v>
       </c>
-      <c r="E33" s="22">
+      <c r="E33" s="21">
         <v>5</v>
       </c>
       <c r="F33"/>
       <c r="G33" s="11">
         <v>1990</v>
       </c>
-      <c r="H33" s="22">
+      <c r="H33" s="21">
         <v>47</v>
       </c>
       <c r="I33"/>
@@ -20568,21 +20840,21 @@
       <c r="A34" s="1">
         <v>2018</v>
       </c>
-      <c r="B34" s="20">
+      <c r="B34" s="23">
         <v>1</v>
       </c>
       <c r="C34"/>
       <c r="D34" s="11">
         <v>2017</v>
       </c>
-      <c r="E34" s="22">
+      <c r="E34" s="21">
         <v>4</v>
       </c>
       <c r="F34"/>
       <c r="G34" s="11">
         <v>2000</v>
       </c>
-      <c r="H34" s="22">
+      <c r="H34" s="21">
         <v>26</v>
       </c>
       <c r="I34"/>
@@ -20596,21 +20868,21 @@
       <c r="A35" s="1">
         <v>2019</v>
       </c>
-      <c r="B35" s="20">
+      <c r="B35" s="23">
         <v>5</v>
       </c>
       <c r="C35"/>
       <c r="D35" s="11">
         <v>2018</v>
       </c>
-      <c r="E35" s="22">
+      <c r="E35" s="21">
         <v>1</v>
       </c>
       <c r="F35"/>
       <c r="G35" s="11">
         <v>2010</v>
       </c>
-      <c r="H35" s="22">
+      <c r="H35" s="21">
         <v>84</v>
       </c>
       <c r="I35"/>
@@ -20624,22 +20896,22 @@
       <c r="A36" s="1">
         <v>2020</v>
       </c>
-      <c r="B36" s="20">
+      <c r="B36" s="23">
         <v>19</v>
       </c>
       <c r="C36"/>
       <c r="D36" s="11">
         <v>2019</v>
       </c>
-      <c r="E36" s="22">
+      <c r="E36" s="21">
         <v>5</v>
       </c>
       <c r="F36"/>
       <c r="G36" s="11">
         <v>2020</v>
       </c>
-      <c r="H36" s="22">
-        <v>145</v>
+      <c r="H36" s="21">
+        <v>147</v>
       </c>
       <c r="I36"/>
       <c r="J36"/>
@@ -20652,22 +20924,22 @@
       <c r="A37" s="1">
         <v>2021</v>
       </c>
-      <c r="B37" s="20">
+      <c r="B37" s="23">
         <v>43</v>
       </c>
       <c r="C37"/>
       <c r="D37" s="11">
         <v>2020</v>
       </c>
-      <c r="E37" s="22">
+      <c r="E37" s="21">
         <v>19</v>
       </c>
       <c r="F37"/>
       <c r="G37" s="12" t="s">
         <v>284</v>
       </c>
-      <c r="H37" s="23">
-        <v>343</v>
+      <c r="H37" s="22">
+        <v>345</v>
       </c>
       <c r="I37"/>
       <c r="J37"/>
@@ -20680,14 +20952,14 @@
       <c r="A38" s="1">
         <v>2022</v>
       </c>
-      <c r="B38" s="20">
+      <c r="B38" s="23">
         <v>9</v>
       </c>
       <c r="C38"/>
       <c r="D38" s="11">
         <v>2021</v>
       </c>
-      <c r="E38" s="22">
+      <c r="E38" s="21">
         <v>43</v>
       </c>
       <c r="F38"/>
@@ -20704,14 +20976,14 @@
       <c r="A39" s="1">
         <v>2023</v>
       </c>
-      <c r="B39" s="20">
+      <c r="B39" s="23">
         <v>25</v>
       </c>
       <c r="C39"/>
       <c r="D39" s="11">
         <v>2022</v>
       </c>
-      <c r="E39" s="22">
+      <c r="E39" s="21">
         <v>9</v>
       </c>
       <c r="F39"/>
@@ -20726,14 +20998,14 @@
       <c r="A40" s="1">
         <v>2024</v>
       </c>
-      <c r="B40" s="20">
+      <c r="B40" s="23">
         <v>14</v>
       </c>
       <c r="C40"/>
       <c r="D40" s="11">
         <v>2023</v>
       </c>
-      <c r="E40" s="22">
+      <c r="E40" s="21">
         <v>25</v>
       </c>
       <c r="F40"/>
@@ -20748,14 +21020,14 @@
       <c r="A41" s="1">
         <v>2025</v>
       </c>
-      <c r="B41" s="20">
+      <c r="B41" s="23">
         <v>31</v>
       </c>
       <c r="C41"/>
       <c r="D41" s="11">
         <v>2024</v>
       </c>
-      <c r="E41" s="22">
+      <c r="E41" s="21">
         <v>14</v>
       </c>
       <c r="F41"/>
@@ -20770,14 +21042,14 @@
       <c r="A42" s="1">
         <v>2026</v>
       </c>
-      <c r="B42" s="20">
-        <v>4</v>
+      <c r="B42" s="23">
+        <v>6</v>
       </c>
       <c r="C42"/>
       <c r="D42" s="11">
         <v>2025</v>
       </c>
-      <c r="E42" s="22">
+      <c r="E42" s="21">
         <v>31</v>
       </c>
       <c r="F42"/>
@@ -20792,15 +21064,15 @@
       <c r="A43" s="1" t="s">
         <v>284</v>
       </c>
-      <c r="B43" s="20">
-        <v>343</v>
+      <c r="B43" s="23">
+        <v>345</v>
       </c>
       <c r="C43"/>
       <c r="D43" s="11">
         <v>2026</v>
       </c>
-      <c r="E43" s="22">
-        <v>4</v>
+      <c r="E43" s="21">
+        <v>6</v>
       </c>
       <c r="F43"/>
       <c r="I43"/>
@@ -20815,8 +21087,8 @@
       <c r="D44" s="12" t="s">
         <v>284</v>
       </c>
-      <c r="E44" s="23">
-        <v>343</v>
+      <c r="E44" s="22">
+        <v>345</v>
       </c>
       <c r="F44"/>
       <c r="I44"/>

</xml_diff>